<commit_message>
Add C2 novelty audit for score invariance and dynamic nonclosure
</commit_message>
<xml_diff>
--- a/docs/editorial/RESULT_CLASSIFICATION.xlsx
+++ b/docs/editorial/RESULT_CLASSIFICATION.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>CLASSICAL ENUMERATION FORMULA; PROJECT CONTRIBUTION IS INDEPENDENT REPRODUCTION AND CORRECTIVE APPLICATION</t>
   </si>
@@ -74,6 +74,90 @@
   </si>
   <si>
     <t>Seek a structural decomposition, recurrence, bounds, or asymptotics for P_n.</t>
+  </si>
+  <si>
+    <t>ELEMENTARY COROLLARY OF STANDARD INTERVAL-SCALE MEASUREMENT INVARIANCE; PROJECT-SPECIFIC CONTEXT FORMULATION</t>
+  </si>
+  <si>
+    <t>Representational measurement theory and meaningful-function functional equations under positive-affine interval-scale transformations</t>
+  </si>
+  <si>
+    <t>C2 COMPLETE — STANDARD INVARIANCE FRAMEWORK FOUND; NO NEED FOR A STRONG NOVELTY CLAIM</t>
+  </si>
+  <si>
+    <t>The project formalizes a short incompatibility among extension stability, numerical positive-affine invariance, continuity, and nontrivial cardinal score differences.</t>
+  </si>
+  <si>
+    <t>A fundamentally new measurement-theory impossibility theorem, or a claim that interval-scale differences are meaningless.</t>
+  </si>
+  <si>
+    <t>DEMOTE TO FOUNDATIONAL LEMMA; KEEP THE CONTEXT–SCALE–CARDINALITY TRILEMMA</t>
+  </si>
+  <si>
+    <t>Cite measurement-invariance literature and state explicitly that numerical invariance is stronger than ordinary scale covariance.</t>
+  </si>
+  <si>
+    <t>CLASSICAL ALGEBRAIC PROPERTY OF THE EXPONENTIAL CERTAINTY EQUIVALENT / ENTROPIC RISK FUNCTIONAL</t>
+  </si>
+  <si>
+    <t>Convex and dynamic entropic risk measures, exponential utility, and log-Laplace transforms</t>
+  </si>
+  <si>
+    <t>C2 COMPLETE — CLASSICAL OBJECT AND DIRECT ALGEBRAIC IDENTITY</t>
+  </si>
+  <si>
+    <t>The framework uses the standard affine covariance Q_lambda(aq+c)=c+a Q_{a lambda}(q) to track score-scale and parameter coupling.</t>
+  </si>
+  <si>
+    <t>A newly discovered log-partition transformation law or evidence for physical renormalization.</t>
+  </si>
+  <si>
+    <t>ATTRIBUTE AS BACKGROUND IDENTITY; RETAIN FOR PARAMETER-STATUS ANALYSIS</t>
+  </si>
+  <si>
+    <t>Cite entropic risk / exponential certainty-equivalent sources in the foundational manuscript.</t>
+  </si>
+  <si>
+    <t>PROJECT-SPECIFIC DIRECT COROLLARY OF CLASSICAL AFFINE COVARIANCE; EXACT BUT NOT AN INDEPENDENT NEW THEOREM</t>
+  </si>
+  <si>
+    <t>Exponential certainty equivalents and affine transformations of log-Laplace functionals</t>
+  </si>
+  <si>
+    <t>C2 COMPLETE — NO IDENTICAL MODEL-SPECIFIC STATEMENT LOCATED; DERIVATION IS ONE-LINE FROM MF-R047</t>
+  </si>
+  <si>
+    <t>For the declared centered contraction, the exact transport law Q'_lambda=(1-a)q_bar+aQ_{a lambda} follows and exposes parameter transport.</t>
+  </si>
+  <si>
+    <t>A previously unknown algebraic identity, a physical evolution law, or a renormalization-group flow.</t>
+  </si>
+  <si>
+    <t>KEEP PROMINENTLY AS CENTRAL EXACT FRAMEWORK PROPOSITION WITH CORRECT ATTRIBUTION</t>
+  </si>
+  <si>
+    <t>Use the identity to introduce the exact non-closure result rather than presenting it as a standalone novelty claim.</t>
+  </si>
+  <si>
+    <t>PROJECT-SPECIFIC EXACT NONCLOSURE COROLLARY WITH AN EXACT FOUR-POINT COUNTEREXAMPLE; NO EXACT PRIOR MATCH FOUND; NOVELTY NOT CERTIFIED</t>
+  </si>
+  <si>
+    <t>Moment-closure hierarchies, sufficient-statistic limitations, and Laplace-transform uniqueness</t>
+  </si>
+  <si>
+    <t>C2 COMPLETE — RELATED GENERAL LITERATURE FOUND, NO EXACT MEAN-PLUS-ONE-Q CLOSURE COUNTEREXAMPLE LOCATED</t>
+  </si>
+  <si>
+    <t>On the unrestricted finite-distribution class, mean plus one fixed-lambda entropic score does not determine the next score; an exact four-point witness is provided.</t>
+  </si>
+  <si>
+    <t>No finite-dimensional closure can exist, the whole curve is always minimal, or the result solves the general moment-closure problem.</t>
+  </si>
+  <si>
+    <t>PROMOTE AS THE STRONGEST SELF-CONTAINED A34 PROPOSITION/COUNTEREXAMPLE</t>
+  </si>
+  <si>
+    <t>Replace numerical matched-state evidence in the main proof with the exact four-point witness; retain broad simulations as support.</t>
   </si>
 </sst>
 </file>
@@ -3548,14 +3632,14 @@
       <c r="H37" s="54" t="str">
         <v>PROVED</v>
       </c>
-      <c r="I37" s="54" t="str">
-        <v>POTENTIALLY ORIGINAL FORMULATION; HIGH-PRIORITY NOVELTY SEARCH</v>
-      </c>
-      <c r="J37" s="54" t="str">
-        <v>Measurement invariance, functional equations, context effects in choice theory</v>
-      </c>
-      <c r="K37" s="54" t="str">
-        <v>DEDICATED NOVELTY SEARCH REQUIRED</v>
+      <c r="I37" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="J37" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="K37" s="54" t="s">
+        <v>23</v>
       </c>
       <c r="L37" s="54" t="str">
         <v>audits/a28_exact_results/a28_theorem.md</v>
@@ -3569,11 +3653,11 @@
       <c r="O37" s="54" t="str">
         <v>The precise continuity, invariance, and extension-stability axioms stated in A28.</v>
       </c>
-      <c r="P37" s="54" t="str">
-        <v>The three audited requirements are jointly incompatible for a nontrivial cardinal score.</v>
-      </c>
-      <c r="Q37" s="54" t="str">
-        <v>No meaningful score can ever be defined, or the theorem applies outside its explicit axioms.</v>
+      <c r="P37" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q37" s="54" t="s">
+        <v>25</v>
       </c>
       <c r="R37" s="54" t="str">
         <v>FOUNDATIONAL NO-GO</v>
@@ -3581,8 +3665,8 @@
       <c r="S37" s="54" t="str">
         <v>FOUNDATIONAL</v>
       </c>
-      <c r="T37" s="54" t="str">
-        <v>PROMOTE TO A CENTRAL THEOREM AFTER LITERATURE REVIEW</v>
+      <c r="T37" s="54" t="s">
+        <v>26</v>
       </c>
       <c r="U37" s="54" t="str">
         <v>P0</v>
@@ -3590,8 +3674,8 @@
       <c r="V37" s="54" t="str">
         <v>IN_REPOSITORY</v>
       </c>
-      <c r="W37" s="54" t="str">
-        <v>Conduct a focused search in measurement theory, quasi-arithmetic means, and context-independent choice.</v>
+      <c r="W37" s="54" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="38">
@@ -4309,14 +4393,14 @@
       <c r="H48" s="54" t="str">
         <v>PROVED ALGEBRAICALLY</v>
       </c>
-      <c r="I48" s="54" t="str">
-        <v>POTENTIALLY ORIGINAL EMPHASIS; ALGEBRA ITSELF ELEMENTARY</v>
-      </c>
-      <c r="J48" s="54" t="str">
-        <v>Log moment-generating functions and entropic risk measures</v>
-      </c>
-      <c r="K48" s="54" t="str">
-        <v>DEDICATED NOVELTY SEARCH REQUIRED</v>
+      <c r="I48" s="54" t="s">
+        <v>28</v>
+      </c>
+      <c r="J48" s="54" t="s">
+        <v>29</v>
+      </c>
+      <c r="K48" s="54" t="s">
+        <v>30</v>
       </c>
       <c r="L48" s="54" t="str">
         <v>audits/a34_exact_results/a34_theorem.md</v>
@@ -4330,11 +4414,11 @@
       <c r="O48" s="54" t="str">
         <v>Fixed positive masses; finite partition sum.</v>
       </c>
-      <c r="P48" s="54" t="str">
-        <v>The scale transformation changes the effective lambda and therefore couples score scale to the parameter.</v>
-      </c>
-      <c r="Q48" s="54" t="str">
-        <v>A physical renormalization-group law.</v>
+      <c r="P48" s="54" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q48" s="54" t="s">
+        <v>32</v>
       </c>
       <c r="R48" s="54" t="str">
         <v>MATHEMATICAL IDENTITY</v>
@@ -4342,8 +4426,8 @@
       <c r="S48" s="54" t="str">
         <v>FOUNDATIONAL</v>
       </c>
-      <c r="T48" s="54" t="str">
-        <v>KEEP AS CORE IDENTITY</v>
+      <c r="T48" s="54" t="s">
+        <v>33</v>
       </c>
       <c r="U48" s="54" t="str">
         <v>P0</v>
@@ -4351,7 +4435,9 @@
       <c r="V48" s="54" t="str">
         <v>IN_REPOSITORY</v>
       </c>
-      <c r="W48" s="54" t="str"/>
+      <c r="W48" s="54" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="56" t="str">
@@ -4378,14 +4464,14 @@
       <c r="H49" s="54" t="str">
         <v>PROVED</v>
       </c>
-      <c r="I49" s="54" t="str">
-        <v>POTENTIALLY ORIGINAL AND TECHNICALLY STRONG; NOVELTY SEARCH REQUIRED</v>
-      </c>
-      <c r="J49" s="54" t="str">
-        <v>Log-Laplace transforms under affine maps; entropic risk measures</v>
-      </c>
-      <c r="K49" s="54" t="str">
-        <v>HIGH-PRIORITY DEDICATED NOVELTY SEARCH</v>
+      <c r="I49" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="J49" s="54" t="s">
+        <v>36</v>
+      </c>
+      <c r="K49" s="54" t="s">
+        <v>37</v>
       </c>
       <c r="L49" s="54" t="str">
         <v>audits/a34_exact_results/a34_theorem.md</v>
@@ -4399,11 +4485,11 @@
       <c r="O49" s="54" t="str">
         <v>Declared centered affine contraction; no general nonlinear dynamics.</v>
       </c>
-      <c r="P49" s="54" t="str">
-        <v>The contraction transports the whole Q(lambda) curve by rescaling lambda.</v>
-      </c>
-      <c r="Q49" s="54" t="str">
-        <v>A fundamental physical evolution equation or closure of the full RZS dynamics.</v>
+      <c r="P49" s="54" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q49" s="54" t="s">
+        <v>39</v>
       </c>
       <c r="R49" s="54" t="str">
         <v>MODEL-SPECIFIC EXACT IDENTITY</v>
@@ -4411,8 +4497,8 @@
       <c r="S49" s="54" t="str">
         <v>FOUNDATIONAL</v>
       </c>
-      <c r="T49" s="54" t="str">
-        <v>PROMOTE TO CENTRAL PROPOSITION AFTER LITERATURE REVIEW</v>
+      <c r="T49" s="54" t="s">
+        <v>40</v>
       </c>
       <c r="U49" s="54" t="str">
         <v>P0</v>
@@ -4420,7 +4506,9 @@
       <c r="V49" s="54" t="str">
         <v>IN_REPOSITORY</v>
       </c>
-      <c r="W49" s="54" t="str"/>
+      <c r="W49" s="54" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="56" t="str">
@@ -4447,14 +4535,14 @@
       <c r="H50" s="54" t="str">
         <v>PROVED</v>
       </c>
-      <c r="I50" s="54" t="str">
-        <v>POTENTIALLY ORIGINAL FRAMEWORK CONSEQUENCE</v>
-      </c>
-      <c r="J50" s="54" t="str">
-        <v>Moment problems, sufficient statistics, closure of log-Laplace transforms</v>
-      </c>
-      <c r="K50" s="54" t="str">
-        <v>DEDICATED NOVELTY SEARCH REQUIRED</v>
+      <c r="I50" s="54" t="s">
+        <v>42</v>
+      </c>
+      <c r="J50" s="54" t="s">
+        <v>43</v>
+      </c>
+      <c r="K50" s="54" t="s">
+        <v>44</v>
       </c>
       <c r="L50" s="54" t="str">
         <v>audits/a34_exact_results/a34_theorem.md</v>
@@ -4468,11 +4556,11 @@
       <c r="O50" s="54" t="str">
         <v>General non-Gaussian microdistributions; specified contraction.</v>
       </c>
-      <c r="P50" s="54" t="str">
-        <v>One point of the Q curve is insufficient for exact dynamics in general.</v>
-      </c>
-      <c r="Q50" s="54" t="str">
-        <v>No finite-dimensional closure can exist under any restricted distribution family.</v>
+      <c r="P50" s="54" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q50" s="54" t="s">
+        <v>46</v>
       </c>
       <c r="R50" s="54" t="str">
         <v>DYNAMIC CLOSURE OBSTRUCTION</v>
@@ -4480,8 +4568,8 @@
       <c r="S50" s="54" t="str">
         <v>FOUNDATIONAL</v>
       </c>
-      <c r="T50" s="54" t="str">
-        <v>KEEP AS CENTRAL THEOREM/COUNTEREXAMPLE</v>
+      <c r="T50" s="54" t="s">
+        <v>47</v>
       </c>
       <c r="U50" s="54" t="str">
         <v>P0</v>
@@ -4489,7 +4577,9 @@
       <c r="V50" s="54" t="str">
         <v>IN_REPOSITORY</v>
       </c>
-      <c r="W50" s="54" t="str"/>
+      <c r="W50" s="54" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="56" t="str">

</xml_diff>